<commit_message>
自動更新 @ 週二 2-25-08 23:01
</commit_message>
<xml_diff>
--- a/detail_giftcode/data/gamedata.xlsx
+++ b/detail_giftcode/data/gamedata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="games" sheetId="1" r:id="rId1"/>
@@ -31280,14 +31280,14 @@
         <v>3561</v>
       </c>
       <c r="F191" s="8" t="str">
-        <f t="shared" ref="F191:F254" si="7">IF(A191="", "", "gift-codes.html?game=" &amp; A191)</f>
-        <v>gift-codes.html?game=手刀搶英雄</v>
+        <f>IF(A191="","", "https://www.ssbuy.tw/detail_giftcode/dist/giftcodes/" &amp; A191 &amp; ".html")</f>
+        <v>https://www.ssbuy.tw/detail_giftcode/dist/giftcodes/手刀搶英雄.html</v>
       </c>
       <c r="G191" s="2" t="s">
         <v>3560</v>
       </c>
       <c r="H191" s="10" t="str">
-        <f t="shared" ref="H191:H254" si="8">IF(A191="", "", "https://www.ssbuy.tw/game-detail.html?game="&amp;A191)</f>
+        <f t="shared" ref="H191:H254" si="7">IF(A191="", "", "https://www.ssbuy.tw/game-detail.html?game="&amp;A191)</f>
         <v>https://www.ssbuy.tw/game-detail.html?game=手刀搶英雄</v>
       </c>
       <c r="I191" s="39" t="s">
@@ -31344,631 +31344,631 @@
     </row>
     <row r="192" spans="1:35" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F192" s="8" t="str">
+        <f t="shared" ref="F191:F254" si="8">IF(A192="", "", "gift-codes.html?game=" &amp; A192)</f>
+        <v/>
+      </c>
+      <c r="H192" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H192" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="193" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F193" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H193" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H193" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="194" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F194" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H194" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H194" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="195" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F195" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H195" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H195" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="196" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F196" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H196" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H196" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="197" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F197" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H197" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H197" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="198" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F198" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H198" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H198" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="199" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F199" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H199" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H199" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="200" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F200" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H200" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H200" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="201" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F201" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H201" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H201" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="202" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F202" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H202" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H202" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="203" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F203" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H203" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H203" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="204" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F204" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H204" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H204" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="205" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F205" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H205" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H205" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="206" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F206" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H206" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H206" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="207" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F207" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H207" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H207" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="208" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F208" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H208" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H208" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="209" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F209" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H209" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H209" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="210" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F210" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H210" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H210" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="211" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F211" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H211" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H211" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="212" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F212" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H212" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H212" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="213" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F213" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H213" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H213" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="214" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F214" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H214" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H214" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="215" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F215" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H215" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H215" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="216" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F216" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H216" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H216" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="217" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F217" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H217" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H217" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="218" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F218" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H218" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H218" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="219" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F219" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H219" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H219" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="220" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F220" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H220" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H220" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="221" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F221" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H221" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H221" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="222" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F222" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H222" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H222" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="223" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F223" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H223" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H223" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="224" spans="6:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F224" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H224" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H224" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="225" spans="6:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F225" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H225" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H225" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="226" spans="6:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F226" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H226" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H226" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="227" spans="6:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F227" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H227" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H227" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="228" spans="6:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F228" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H228" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H228" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="229" spans="6:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F229" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H229" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H229" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="230" spans="6:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F230" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H230" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H230" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="231" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F231" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H231" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H231" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="232" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F232" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H232" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H232" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="233" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F233" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H233" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H233" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="234" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F234" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H234" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H234" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="235" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F235" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H235" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H235" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="236" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F236" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H236" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H236" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="237" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F237" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H237" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H237" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="238" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F238" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H238" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H238" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="239" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F239" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H239" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H239" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="240" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F240" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H240" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H240" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="241" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F241" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H241" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H241" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="242" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F242" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H242" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H242" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="243" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F243" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H243" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H243" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="244" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F244" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H244" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H244" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="245" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F245" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H245" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H245" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="246" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F246" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H246" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H246" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="247" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F247" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H247" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H247" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="248" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F248" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H248" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H248" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="249" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F249" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H249" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H249" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="250" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F250" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H250" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H250" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="251" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F251" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H251" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H251" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="252" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F252" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H252" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H252" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="253" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F253" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H253" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H253" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="254" spans="6:8" ht="19.5" x14ac:dyDescent="0.25">
       <c r="F254" s="8" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="H254" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H254" s="10" t="str">
-        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
自動更新 @ 週三 2-25-08 00:08
</commit_message>
<xml_diff>
--- a/detail_giftcode/data/gamedata.xlsx
+++ b/detail_giftcode/data/gamedata.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5487" uniqueCount="3681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5528" uniqueCount="3713">
   <si>
     <t>Facebook</t>
   </si>
@@ -15040,6 +15040,253 @@
   <si>
     <t>封神：蒼嵐契約</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gear Fight!</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://apps.apple.com/tw/app/gear-fight/id6738430824</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.EternalStudio.GearFight&amp;hl=zh_TW</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://voodoo.io/</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.facebook.com/</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>《</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Gear Fight</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>》是一款考驗策略與創造力的益智冒險手遊。玩家將化身為機械大師，親手設計戰爭機器，透過巧妙組合、放置齒輪，打造出獨一無二的自動化生產線來抵禦強敵。你需要在有限預算內，策略性地生產近戰兵、弓箭手等多樣單位。為了讓你的開局更順利，記得隨時搜尋最新的禮包碼來兌換豐厚獎勵；若想加速升級，安全的代儲值服務是你的最佳幫手，讓你輕鬆構築最強工廠，迎向勝利。</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>700寶石</t>
+  </si>
+  <si>
+    <t>200寶石</t>
+  </si>
+  <si>
+    <t>25寶石</t>
+  </si>
+  <si>
+    <t>2X加速</t>
+  </si>
+  <si>
+    <t>植物部隊包</t>
+  </si>
+  <si>
+    <t>祝福禮包</t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.gamania.tosm&amp;is_retargeting=true&amp;source_caller=ui&amp;shortlink=tr8m0yil&amp;c=0715preregister&amp;pid=pre-eventpage_registernowbtn&amp;af_xp=custom&amp;fbclid=IwY2xjawMat9dleHRuA2FlbQIxMABicmlkETFQdUxnS1dmdVZuODkyZWp0AR6xAzlsZNQNCXjTWaD3u5fhy0zWK0zT2-hw23w4-G2KqEx0eosDi8BsaQWa8w_aem_pSu3Tr4ufEnibbPRTHgBGw&amp;af_reengagement_window=61d</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>救世者之樹 M</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://apps.apple.com/tw/app/%E6%95%91%E4%B8%96%E8%80%85%E4%B9%8B%E6%A8%B9%EF%BD%8D/id6458050011</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://tosm-treeofsavior.beanfun.com/main</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.facebook.com/TreeofSaviorM/</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>《救世者之樹</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>》是經典</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>線上遊戲《救世者之樹》的全新</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>MMORPG</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>手機版，完美繼承了其獨樹一幟的童話繪本美術風格。遊戲以精緻的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>3D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>場景搭配經典的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>角色，帶領玩家重溫最初的感動。遊戲提供劍士、巫師、弓箭手、牧師四大經典職業體系，玩家可以自由搭配技能與特性，打造專屬於你的獨特玩法。除了豐富的主線劇情，還有特色的「夥伴」系統與「隨機副本」等著你來探索。為了讓你的冒險旅程更加順利，記得隨時關注官方釋出的最新禮包碼，兌換豐富的開服好禮。此外，透過方便安全的代儲值服務，也能幫助你快速成長，讓角色戰力快人一步，輕鬆挑戰更高難度的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>BOSS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="細明體"/>
+        <family val="3"/>
+        <charset val="136"/>
+      </rPr>
+      <t>。</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>R1F437D9FA</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TP禮包</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>主畫面中按設定/個人頭像</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>找到兌換碼禮包碼字樣點進去</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>按確定後到信箱領取免費禮包</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1500TP</t>
+  </si>
+  <si>
+    <t>1150TP</t>
+  </si>
+  <si>
+    <t>580TP</t>
+  </si>
+  <si>
+    <t>350TP</t>
+  </si>
+  <si>
+    <t>165TP</t>
+  </si>
+  <si>
+    <t>80TP</t>
+  </si>
+  <si>
+    <t>40TP</t>
+  </si>
+  <si>
+    <t>13TP</t>
+  </si>
+  <si>
+    <t>TOSM上市新手禮包</t>
   </si>
 </sst>
 </file>
@@ -32468,24 +32715,150 @@
         <v>391</v>
       </c>
     </row>
-    <row r="198" spans="1:33" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:33" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="1" t="s">
+        <v>3681</v>
+      </c>
+      <c r="C198" s="1" t="s">
+        <v>3685</v>
+      </c>
+      <c r="D198" s="23" t="s">
+        <v>3684</v>
+      </c>
+      <c r="E198" s="23" t="s">
+        <v>3682</v>
+      </c>
       <c r="F198" s="8" t="str">
         <f t="shared" si="8"/>
-        <v/>
+        <v>gift-codes.html?game=Gear Fight!</v>
+      </c>
+      <c r="G198" s="23" t="s">
+        <v>3683</v>
       </c>
       <c r="H198" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-    </row>
-    <row r="199" spans="1:33" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>https://www.ssbuy.tw/game-detail.html?game=Gear Fight!</v>
+      </c>
+      <c r="I198" s="39" t="s">
+        <v>3686</v>
+      </c>
+      <c r="J198" s="3" t="s">
+        <v>3687</v>
+      </c>
+      <c r="K198" s="4">
+        <v>780</v>
+      </c>
+      <c r="L198" s="3" t="s">
+        <v>3688</v>
+      </c>
+      <c r="M198" s="4">
+        <v>232</v>
+      </c>
+      <c r="N198" s="3" t="s">
+        <v>3689</v>
+      </c>
+      <c r="O198" s="4">
+        <v>51</v>
+      </c>
+      <c r="P198" s="3" t="s">
+        <v>3690</v>
+      </c>
+      <c r="Q198" s="4">
+        <v>232</v>
+      </c>
+      <c r="R198" s="3" t="s">
+        <v>3691</v>
+      </c>
+      <c r="S198" s="4">
+        <v>391</v>
+      </c>
+      <c r="T198" s="3" t="s">
+        <v>3692</v>
+      </c>
+      <c r="U198" s="4">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="199" spans="1:33" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="22" t="s">
+        <v>3694</v>
+      </c>
+      <c r="C199" s="24" t="s">
+        <v>3697</v>
+      </c>
+      <c r="D199" s="23" t="s">
+        <v>3696</v>
+      </c>
+      <c r="E199" s="23" t="s">
+        <v>3695</v>
+      </c>
       <c r="F199" s="8" t="str">
         <f t="shared" si="8"/>
-        <v/>
+        <v>gift-codes.html?game=救世者之樹 M</v>
+      </c>
+      <c r="G199" s="23" t="s">
+        <v>3693</v>
       </c>
       <c r="H199" s="10" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v>https://www.ssbuy.tw/game-detail.html?game=救世者之樹 M</v>
+      </c>
+      <c r="I199" s="39" t="s">
+        <v>3698</v>
+      </c>
+      <c r="J199" s="3" t="s">
+        <v>3704</v>
+      </c>
+      <c r="K199" s="4">
+        <v>2555</v>
+      </c>
+      <c r="L199" s="3" t="s">
+        <v>3705</v>
+      </c>
+      <c r="M199" s="4">
+        <v>2119</v>
+      </c>
+      <c r="N199" s="3" t="s">
+        <v>3706</v>
+      </c>
+      <c r="O199" s="4">
+        <v>1063</v>
+      </c>
+      <c r="P199" s="3" t="s">
+        <v>3707</v>
+      </c>
+      <c r="Q199" s="4">
+        <v>701</v>
+      </c>
+      <c r="R199" s="3" t="s">
+        <v>3708</v>
+      </c>
+      <c r="S199" s="4">
+        <v>312</v>
+      </c>
+      <c r="T199" s="3" t="s">
+        <v>3709</v>
+      </c>
+      <c r="U199" s="4">
+        <v>162</v>
+      </c>
+      <c r="V199" s="3" t="s">
+        <v>3710</v>
+      </c>
+      <c r="W199" s="4">
+        <v>85</v>
+      </c>
+      <c r="X199" s="3" t="s">
+        <v>3711</v>
+      </c>
+      <c r="Y199" s="4">
+        <v>51</v>
+      </c>
+      <c r="Z199" s="3" t="s">
+        <v>3712</v>
+      </c>
+      <c r="AA199" s="4">
+        <v>654</v>
       </c>
     </row>
     <row r="200" spans="1:33" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -36663,9 +37036,16 @@
     <hyperlink ref="G195" r:id="rId54"/>
     <hyperlink ref="D196" r:id="rId55"/>
     <hyperlink ref="G197" r:id="rId56"/>
+    <hyperlink ref="E198" r:id="rId57"/>
+    <hyperlink ref="G198" r:id="rId58"/>
+    <hyperlink ref="D198" r:id="rId59"/>
+    <hyperlink ref="G199"/>
+    <hyperlink ref="E199" r:id="rId60"/>
+    <hyperlink ref="D199" r:id="rId61"/>
+    <hyperlink ref="C199" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId57"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId63"/>
 </worksheet>
 </file>
 
@@ -49071,37 +49451,73 @@
     <row r="198" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="49" t="str">
         <f>IF(games!A198="", "", games!A198)</f>
-        <v/>
+        <v>Gear Fight!</v>
       </c>
       <c r="C198" s="49" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v>giftcodesbanner/Gear Fight!-禮包碼.jpg</v>
       </c>
       <c r="D198" s="49" t="str">
         <f t="shared" si="8"/>
-        <v/>
+        <v>https://www.ssbuy.tw/gift-codes.html?game=Gear Fight!</v>
       </c>
       <c r="E198" s="50" t="str">
         <f>IF(games!I198&lt;&gt;"", games!I198, "")</f>
-        <v/>
+        <v>《Gear Fight》是一款考驗策略與創造力的益智冒險手遊。玩家將化身為機械大師，親手設計戰爭機器，透過巧妙組合、放置齒輪，打造出獨一無二的自動化生產線來抵禦強敵。你需要在有限預算內，策略性地生產近戰兵、弓箭手等多樣單位。為了讓你的開局更順利，記得隨時搜尋最新的禮包碼來兌換豐厚獎勵；若想加速升級，安全的代儲值服務是你的最佳幫手，讓你輕鬆構築最強工廠，迎向勝利。</v>
+      </c>
+      <c r="F198" s="53" t="s">
+        <v>2666</v>
+      </c>
+      <c r="G198" s="49" t="s">
+        <v>2666</v>
+      </c>
+      <c r="H198" s="54" t="s">
+        <v>2666</v>
+      </c>
+      <c r="I198" s="49" t="s">
+        <v>2666</v>
+      </c>
+      <c r="K198" s="53" t="s">
+        <v>2666</v>
+      </c>
+      <c r="L198" s="49" t="s">
+        <v>2666</v>
+      </c>
+      <c r="M198" s="54" t="s">
+        <v>2666</v>
+      </c>
+      <c r="N198" s="49" t="s">
+        <v>2666</v>
       </c>
     </row>
     <row r="199" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="49" t="str">
         <f>IF(games!A199="", "", games!A199)</f>
-        <v/>
+        <v>救世者之樹 M</v>
       </c>
       <c r="C199" s="49" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v>giftcodesbanner/救世者之樹 M-禮包碼.jpg</v>
       </c>
       <c r="D199" s="49" t="str">
         <f t="shared" si="8"/>
-        <v/>
+        <v>https://www.ssbuy.tw/gift-codes.html?game=救世者之樹 M</v>
       </c>
       <c r="E199" s="50" t="str">
         <f>IF(games!I199&lt;&gt;"", games!I199, "")</f>
-        <v/>
+        <v>《救世者之樹 M》是經典PC線上遊戲《救世者之樹》的全新MMORPG手機版，完美繼承了其獨樹一幟的童話繪本美術風格。遊戲以精緻的3D場景搭配經典的2D角色，帶領玩家重溫最初的感動。遊戲提供劍士、巫師、弓箭手、牧師四大經典職業體系，玩家可以自由搭配技能與特性，打造專屬於你的獨特玩法。除了豐富的主線劇情，還有特色的「夥伴」系統與「隨機副本」等著你來探索。為了讓你的冒險旅程更加順利，記得隨時關注官方釋出的最新禮包碼，兌換豐富的開服好禮。此外，透過方便安全的代儲值服務，也能幫助你快速成長，讓角色戰力快人一步，輕鬆挑戰更高難度的BOSS。</v>
+      </c>
+      <c r="F199" s="70" t="s">
+        <v>3701</v>
+      </c>
+      <c r="G199" s="49" t="s">
+        <v>3702</v>
+      </c>
+      <c r="H199" s="49" t="s">
+        <v>2651</v>
+      </c>
+      <c r="I199" s="49" t="s">
+        <v>3703</v>
       </c>
     </row>
     <row r="200" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -49120,6 +49536,12 @@
       <c r="E200" s="50" t="str">
         <f>IF(games!I200&lt;&gt;"", games!I200, "")</f>
         <v/>
+      </c>
+      <c r="K200" s="53" t="s">
+        <v>3699</v>
+      </c>
+      <c r="L200" s="49" t="s">
+        <v>3700</v>
       </c>
     </row>
     <row r="201" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
自動更新 @ 週三 2-25-08 21:11
</commit_message>
<xml_diff>
--- a/detail_giftcode/data/gamedata.xlsx
+++ b/detail_giftcode/data/gamedata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="games" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5528" uniqueCount="3713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5544" uniqueCount="3722">
   <si>
     <t>Facebook</t>
   </si>
@@ -15287,6 +15287,42 @@
   </si>
   <si>
     <t>TOSM上市新手禮包</t>
+  </si>
+  <si>
+    <t>GOBLIN0820STRONG</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>fanghuo</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>金幣與強化禮包</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>94AKAONI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>94DADA</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>RCB768501E</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>94MMD</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>B156BCDGBF</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>OB1CE9EJ5F</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -48789,6 +48825,12 @@
       <c r="N185" s="49" t="s">
         <v>2658</v>
       </c>
+      <c r="O185" s="54" t="s">
+        <v>3714</v>
+      </c>
+      <c r="P185" s="49" t="s">
+        <v>3715</v>
+      </c>
     </row>
     <row r="186" spans="1:50" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="79" t="s">
@@ -49519,6 +49561,54 @@
       <c r="I199" s="49" t="s">
         <v>3703</v>
       </c>
+      <c r="K199" s="53" t="s">
+        <v>3699</v>
+      </c>
+      <c r="L199" s="49" t="s">
+        <v>3700</v>
+      </c>
+      <c r="M199" s="54" t="s">
+        <v>3713</v>
+      </c>
+      <c r="N199" s="49" t="s">
+        <v>3700</v>
+      </c>
+      <c r="O199" s="66" t="s">
+        <v>3718</v>
+      </c>
+      <c r="P199" s="49" t="s">
+        <v>3700</v>
+      </c>
+      <c r="Q199" s="66" t="s">
+        <v>3716</v>
+      </c>
+      <c r="R199" s="49" t="s">
+        <v>3700</v>
+      </c>
+      <c r="S199" s="54" t="s">
+        <v>3717</v>
+      </c>
+      <c r="T199" s="49" t="s">
+        <v>3700</v>
+      </c>
+      <c r="U199" s="54" t="s">
+        <v>3719</v>
+      </c>
+      <c r="V199" s="49" t="s">
+        <v>3700</v>
+      </c>
+      <c r="W199" s="54" t="s">
+        <v>3720</v>
+      </c>
+      <c r="X199" s="49" t="s">
+        <v>3700</v>
+      </c>
+      <c r="Y199" s="54" t="s">
+        <v>3721</v>
+      </c>
+      <c r="Z199" s="49" t="s">
+        <v>3700</v>
+      </c>
     </row>
     <row r="200" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="49" t="str">
@@ -49536,12 +49626,6 @@
       <c r="E200" s="50" t="str">
         <f>IF(games!I200&lt;&gt;"", games!I200, "")</f>
         <v/>
-      </c>
-      <c r="K200" s="53" t="s">
-        <v>3699</v>
-      </c>
-      <c r="L200" s="49" t="s">
-        <v>3700</v>
       </c>
     </row>
     <row r="201" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>